<commit_message>
small fixes and enhancements
</commit_message>
<xml_diff>
--- a/batch_dcf_output.xlsx
+++ b/batch_dcf_output.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Financials" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projections (Base Case)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qualitative Insights" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +39,15 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,13 +77,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,7 +498,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -505,21 +523,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Target Price (Perp. Growth)</t>
+          <t>Implied Share Price (DCF)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>0</v>
+        <v>261.802579346862</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Target Price (Exit Multiple)</t>
+          <t>Implied Share Price (Exit Multiple)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>0</v>
+        <v>227.5192230668335</v>
       </c>
     </row>
     <row r="12">
@@ -537,28 +555,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Target Price (Perp. Growth)</t>
+          <t>Implied Share Price (DCF)</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>361.8245677643</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Target Price (Exit Multiple)</t>
+          <t>Implied Share Price (Exit Multiple)</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0</v>
+        <v>311.9671873635205</v>
       </c>
     </row>
     <row r="17">
@@ -576,28 +594,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Target Price (Perp. Growth)</t>
+          <t>Implied Share Price (DCF)</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>0</v>
+        <v>514.3472071209335</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Target Price (Exit Multiple)</t>
+          <t>Implied Share Price (Exit Multiple)</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>0</v>
+        <v>440.2473654287473</v>
       </c>
     </row>
     <row r="22">
@@ -610,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Given the lack of forward-looking assumptions provided by management, and considering only historical data which shows no revenue for the years from 2020 to 2025, a base case scenario is assumed with zero growth. Bear and Bull scenarios are estimated based on typical market volatility but without specific information, these are speculative.</t>
+          <t>The revenue has been declining significantly over the past few years, with a sharp drop from 2021 to 2022 and an increase in 2025 that is not substantiated by forward-looking assumptions.</t>
         </is>
       </c>
     </row>
@@ -625,10 +643,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -681,22 +699,22 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>0</v>
+        <v>47468000</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>0</v>
+        <v>41436000</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>368161</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0</v>
+        <v>373355</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0</v>
+        <v>155584</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0</v>
+        <v>704326</v>
       </c>
     </row>
     <row r="3">
@@ -706,22 +724,22 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>58822</v>
+        <v>47468000</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0</v>
+        <v>41436000</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0</v>
+        <v>368159</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0</v>
+        <v>373278</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>59281</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>136717</v>
+        <v>704326</v>
       </c>
     </row>
     <row r="4">
@@ -731,22 +749,22 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0</v>
+        <v>-4391000</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0</v>
+        <v>-13045000</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0</v>
+        <v>16663</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0</v>
+        <v>18079</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>334</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0</v>
+        <v>26556</v>
       </c>
     </row>
     <row r="5">
@@ -756,6 +774,383 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
+        <v>32804000</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>29825000</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>17139</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>10149</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>10149</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>86501</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>176912000</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>290461000</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>308079</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>311276</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>437560</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>575938</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Total Debt</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>82793000</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>59383000</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>60541</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>45254000</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>108282000</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>174647</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Operating Cash Flow</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>33319000</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>33319000</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-10262</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>50424</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>155584</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>172767</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CapEx</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>-20402000</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-28458000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>-35597</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>--- ML Features (KPIs) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>EBIT Margin</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.9999945675940689</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.9997937619691715</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.381022470176882</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Net Margin</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.6910760933681638</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.7197847282556231</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.04655300262656827</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.02718324382959917</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0.06523164335664336</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0.1228138674420652</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>CapEx / Revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>-0.4298053425465577</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>-0.6867940920938315</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>-0.2287960201563143</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>ROA (Net Income / Assets)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.1854255222935697</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.1026815992508461</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.05563183469175114</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.03260450532646269</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0.02319453332114453</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>0.1501915136698742</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Projected Year 1</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Projected Year 2</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Projected Year 3</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Projected Year 4</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Projected Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>683196220</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>662700333.4</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>642819323.398</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>623534743.6960599</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>604828701.3851781</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>683196220</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>662700333.4</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>642819323.398</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>623534743.6960599</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>604828701.3851781</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D&amp;A</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>25759320</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>24986540.4</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>24236944.188</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>23509835.86236</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>22804540.78648919</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>CapEx</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="5" t="n">
@@ -770,133 +1165,137 @@
       <c r="F5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Total Assets</t>
+          <t>Unlevered Free Cash Flow</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0</v>
+        <v>538156485</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>290461</v>
+        <v>522011790.4499999</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0</v>
+        <v>506351436.7365</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>491160893.634405</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>575938</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Total Debt</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>476426066.8253728</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Operating Cash Flow</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>29825</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>172767</v>
+          <t>--- Projected ML Features ---</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>CapEx</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>364</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>348</v>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>EBIT Margin</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>UFCF Margin</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.7877041313255509</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.7877041313255508</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.7877041313255509</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.7877041313255509</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0.7877041313255509</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AI Qualitative Management Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Management Confidence Score (1-10):</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Confidence Rationale:</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Management does not provide any forward-looking revenue growth projections or specific strategies, indicating a lack of confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Overall Insight Summary:</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The revenue has been declining significantly over the past few years, with a sharp drop from 2021 to 2022 and an increase in 2025 that is not substantiated by forward-looking assumptions.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more updte and finishn of the phase 3
</commit_message>
<xml_diff>
--- a/batch_dcf_output.xlsx
+++ b/batch_dcf_output.xlsx
@@ -44,7 +44,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
   </fonts>
   <fills count="4">
@@ -475,7 +475,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>VH2.DE</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8.26%</t>
+          <t>9.27%</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-10.00%</t>
+          <t>2.00%</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>261.802579346862</v>
+        <v>90.70847494686804</v>
       </c>
     </row>
     <row r="10">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>227.5192230668335</v>
+        <v>93.6685782031622</v>
       </c>
     </row>
     <row r="12">
@@ -555,7 +555,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-3.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>361.8245677643</v>
+        <v>103.6307950021277</v>
       </c>
     </row>
     <row r="15">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>311.9671873635205</v>
+        <v>107.0525782612467</v>
       </c>
     </row>
     <row r="17">
@@ -594,7 +594,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>8.00%</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>514.3472071209335</v>
+        <v>118.01144038406</v>
       </c>
     </row>
     <row r="20">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>440.2473654287473</v>
+        <v>121.9507922975198</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>The revenue has been declining significantly over the past few years, with a sharp drop from 2021 to 2022 and an increase in 2025 that is not substantiated by forward-looking assumptions.</t>
+          <t>Fallback to static rates due to error.</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -651,8 +651,6 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,30 +661,20 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Year 2020</t>
+          <t>Year 2022</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Year 2021</t>
+          <t>Year 2023</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Year 2022</t>
+          <t>Year 2024</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Year 2023</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Year 2024</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Year 2025</t>
         </is>
@@ -699,22 +687,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>47468000</v>
+        <v>394328000000</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>41436000</v>
+        <v>383285000000</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>368161</v>
+        <v>391035000000</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>373355</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>155584</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>704326</v>
+        <v>416161000000</v>
       </c>
     </row>
     <row r="3">
@@ -724,22 +706,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>47468000</v>
+        <v>119437000000</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>41436000</v>
+        <v>114301000000</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>368159</v>
+        <v>123216000000</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>373278</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>59281</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>704326</v>
+        <v>133050000000</v>
       </c>
     </row>
     <row r="4">
@@ -749,22 +725,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>-4391000</v>
+        <v>11104000000</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>-13045000</v>
+        <v>11519000000</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>16663</v>
+        <v>11445000000</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>18079</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>334</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>26556</v>
+        <v>11698000000</v>
       </c>
     </row>
     <row r="5">
@@ -774,22 +744,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>32804000</v>
+        <v>99803000000</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>29825000</v>
+        <v>96995000000</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>17139</v>
+        <v>93736000000</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>10149</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>10149</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>86501</v>
+        <v>112010000000</v>
       </c>
     </row>
     <row r="6">
@@ -799,22 +763,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>176912000</v>
+        <v>352755000000</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>290461000</v>
+        <v>352583000000</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>308079</v>
+        <v>364980000000</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>311276</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>437560</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>575938</v>
+        <v>359241000000</v>
       </c>
     </row>
     <row r="7">
@@ -824,22 +782,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>82793000</v>
+        <v>132480000000</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>59383000</v>
+        <v>111088000000</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0</v>
+        <v>106629000000</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>60541</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>0</v>
+        <v>98657000000</v>
       </c>
     </row>
     <row r="8">
@@ -849,22 +801,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>45254000</v>
+        <v>23646000000</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>108282000</v>
+        <v>29965000000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>31</v>
+        <v>29943000000</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>174647</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>22</v>
+        <v>35934000000</v>
       </c>
     </row>
     <row r="9">
@@ -874,22 +820,16 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>33319000</v>
+        <v>122151000000</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>33319000</v>
+        <v>110543000000</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>-10262</v>
+        <v>118254000000</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>50424</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>155584</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>172767</v>
+        <v>111482000000</v>
       </c>
     </row>
     <row r="10">
@@ -899,22 +839,16 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>-20402000</v>
+        <v>10708000000</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>-28458000</v>
+        <v>10959000000</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0</v>
+        <v>9447000000</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>-35597</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>0</v>
+        <v>12715000000</v>
       </c>
     </row>
     <row r="13">
@@ -931,22 +865,16 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1</v>
+        <v>0.3028874439552859</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1</v>
+        <v>0.2982141226502472</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>0.9999945675940689</v>
+        <v>0.3151022287007557</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0.9997937619691715</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0.381022470176882</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
     </row>
     <row r="15">
@@ -956,22 +884,16 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>0.6910760933681638</v>
+        <v>0.2530964070519973</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>0.7197847282556231</v>
+        <v>0.2530623426432028</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>0.04655300262656827</v>
+        <v>0.2397125576994387</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02718324382959917</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>0.06523164335664336</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>0.1228138674420652</v>
+        <v>0.2691506412181824</v>
       </c>
     </row>
     <row r="16">
@@ -981,22 +903,16 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>-0.4298053425465577</v>
+        <v>0.02715505873283155</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>-0.6867940920938315</v>
+        <v>0.02859230076835775</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0</v>
+        <v>0.02415896275269477</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>-0.2287960201563143</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>0</v>
+        <v>0.03055307921693768</v>
       </c>
     </row>
     <row r="17">
@@ -1006,22 +922,16 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>0.1854255222935697</v>
+        <v>0.2829244092925685</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0.1026815992508461</v>
+        <v>0.2750983456377648</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0.05563183469175114</v>
+        <v>0.2568250315085758</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.03260450532646269</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>0.02319453332114453</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>0.1501915136698742</v>
+        <v>0.3117962593356549</v>
       </c>
     </row>
   </sheetData>
@@ -1085,19 +995,19 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>683196220</v>
+        <v>436969050000</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>662700333.4</v>
+        <v>458817502500</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>642819323.398</v>
+        <v>481758377625.0001</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>623534743.6960599</v>
+        <v>505846296506.2501</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>604828701.3851781</v>
+        <v>531138611331.5626</v>
       </c>
     </row>
     <row r="3">
@@ -1107,19 +1017,19 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>683196220</v>
+        <v>139702500000</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>662700333.4</v>
+        <v>146687625000</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>642819323.398</v>
+        <v>154022006250</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>623534743.6960599</v>
+        <v>161723106562.5001</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>604828701.3851781</v>
+        <v>169809261890.6251</v>
       </c>
     </row>
     <row r="4">
@@ -1129,19 +1039,19 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>25759320</v>
+        <v>12282900000</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>24986540.4</v>
+        <v>12897045000</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>24236944.188</v>
+        <v>13541897250</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>23509835.86236</v>
+        <v>14218992112.5</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>22804540.78648919</v>
+        <v>14929941718.125</v>
       </c>
     </row>
     <row r="5">
@@ -1151,19 +1061,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0</v>
+        <v>13350750000</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0</v>
+        <v>14018287500</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0</v>
+        <v>14719201875</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0</v>
+        <v>15455161968.75</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>16227920067.1875</v>
       </c>
     </row>
     <row r="6">
@@ -1173,19 +1083,19 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>538156485</v>
+        <v>103709025000</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>522011790.4499999</v>
+        <v>108894476250</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>506351436.7365</v>
+        <v>114339200062.5</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>491160893.634405</v>
+        <v>120056160065.625</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>476426066.8253728</v>
+        <v>126058968068.9063</v>
       </c>
     </row>
     <row r="9">
@@ -1202,19 +1112,19 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1</v>
+        <v>0.3197079976259188</v>
       </c>
     </row>
     <row r="11">
@@ -1224,19 +1134,19 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>0.7877041313255509</v>
+        <v>0.2373372324653199</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.7877041313255508</v>
+        <v>0.2373372324653199</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.7877041313255509</v>
+        <v>0.23733723246532</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.7877041313255509</v>
+        <v>0.23733723246532</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.7877041313255509</v>
+        <v>0.23733723246532</v>
       </c>
     </row>
   </sheetData>
@@ -1271,7 +1181,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1282,7 +1192,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Management does not provide any forward-looking revenue growth projections or specific strategies, indicating a lack of confidence.</t>
+          <t>Failed to parse LLM insight.</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1204,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The revenue has been declining significantly over the past few years, with a sharp drop from 2021 to 2022 and an increase in 2025 that is not substantiated by forward-looking assumptions.</t>
+          <t>Fallback to static rates due to error.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
try to fill all the ticers
</commit_message>
<xml_diff>
--- a/batch_dcf_output.xlsx
+++ b/batch_dcf_output.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>HOG</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14.35%</t>
+          <t>10.16%</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>-7.60493113167658</v>
+        <v>46.92594593674662</v>
       </c>
     </row>
     <row r="10">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>8.572395959018873</v>
+        <v>58.69387983101826</v>
       </c>
     </row>
     <row r="12">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>-7.791132397288223</v>
+        <v>53.16056752434386</v>
       </c>
     </row>
     <row r="15">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>10.90933249309379</v>
+        <v>66.76391703866112</v>
       </c>
     </row>
     <row r="17">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>-7.997344052484059</v>
+        <v>60.09272318802731</v>
       </c>
     </row>
     <row r="20">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>13.53169696792239</v>
+        <v>75.75367447589016</v>
       </c>
     </row>
     <row r="22">
@@ -687,16 +687,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>63054000000</v>
+        <v>5755130000</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>54228000000</v>
+        <v>5836478000</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>53101000000</v>
+        <v>5186802000</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>52853000000</v>
+        <v>4473175000</v>
       </c>
     </row>
     <row r="3">
@@ -706,16 +706,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>8264000000</v>
+        <v>962468000</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1640000000</v>
+        <v>897663000</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>-10176000000</v>
+        <v>547886000</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2648000000</v>
+        <v>492175000</v>
       </c>
     </row>
     <row r="4">
@@ -725,16 +725,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>13035000000</v>
+        <v>151942000</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>9602000000</v>
+        <v>158112000</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>11379000000</v>
+        <v>160673000</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>11706000000</v>
+        <v>172371000</v>
       </c>
     </row>
     <row r="5">
@@ -744,16 +744,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>8014000000</v>
+        <v>741408000</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>1689000000</v>
+        <v>706586000</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>-18756000000</v>
+        <v>455357000</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-267000000</v>
+        <v>338738000</v>
       </c>
     </row>
     <row r="6">
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>182103000000</v>
+        <v>11492476000</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>191572000000</v>
+        <v>12140554000</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>196485000000</v>
+        <v>11881579000</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>211429000000</v>
+        <v>8044815000</v>
       </c>
     </row>
     <row r="7">
@@ -782,16 +782,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>42007000000</v>
+        <v>6955287000</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>49266000000</v>
+        <v>7196053000</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>50011000000</v>
+        <v>7026460000</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>46585000000</v>
+        <v>3053696000</v>
       </c>
     </row>
     <row r="8">
@@ -801,16 +801,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11144000000</v>
+        <v>1433175000</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>7079000000</v>
+        <v>1533806000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>8249000000</v>
+        <v>1589608000</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>14265000000</v>
+        <v>3091744000</v>
       </c>
     </row>
     <row r="9">
@@ -820,16 +820,16 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>15433000000</v>
+        <v>548461000</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>11471000000</v>
+        <v>754887000</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>8288000000</v>
+        <v>1063833000</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>9697000000</v>
+        <v>568922000</v>
       </c>
     </row>
     <row r="10">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>24844000000</v>
+        <v>151669000</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>25750000000</v>
+        <v>207404000</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>23944000000</v>
+        <v>196563000</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>14646000000</v>
+        <v>153679000</v>
       </c>
     </row>
     <row r="13">
@@ -865,16 +865,16 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>0.1310622640910965</v>
+        <v>0.1672365350565495</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>0.03024267905878882</v>
+        <v>0.1538021731599091</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>-0.1916348091373044</v>
+        <v>0.1056307913816645</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
     </row>
     <row r="15">
@@ -884,16 +884,16 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>0.1270974085704317</v>
+        <v>0.1288255869111558</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>0.03114627129895995</v>
+        <v>0.1210637648252936</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>-0.3532136871245363</v>
+        <v>0.08779147536381762</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>-0.005051747299112633</v>
+        <v>0.07572652534273754</v>
       </c>
     </row>
     <row r="16">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>0.3940114822215878</v>
+        <v>0.02635370530292105</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>0.4748469425389098</v>
+        <v>0.03553581457858661</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0.4509142953993334</v>
+        <v>0.03789676181971088</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0.2771082057782907</v>
+        <v>0.03435568695613295</v>
       </c>
     </row>
     <row r="17">
@@ -922,16 +922,16 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>0.04400806137186098</v>
+        <v>0.06451246885353513</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0.008816528511473493</v>
+        <v>0.05820047421229706</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>-0.09545766852431484</v>
+        <v>0.038324619985273</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-0.001262835278036599</v>
+        <v>0.04210637534859409</v>
       </c>
     </row>
   </sheetData>
@@ -995,19 +995,19 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>55495650000</v>
+        <v>4696833750</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>58270432500</v>
+        <v>4931675437.5</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>61183954125.00001</v>
+        <v>5178259209.375001</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>64243151831.25002</v>
+        <v>5437172169.843751</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>67455309422.81252</v>
+        <v>5709030778.335939</v>
       </c>
     </row>
     <row r="3">
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>2780400000</v>
+        <v>516783750.0000001</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>2919420000</v>
+        <v>542622937.5</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>3065391000</v>
+        <v>569754084.3750001</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>3218660550.000001</v>
+        <v>598241788.5937501</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>3379593577.500001</v>
+        <v>628153878.0234377</v>
       </c>
     </row>
     <row r="4">
@@ -1039,19 +1039,19 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>12291300000</v>
+        <v>180989550</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>12905865000</v>
+        <v>190039027.5</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>13551158250</v>
+        <v>199540978.875</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>14228716162.5</v>
+        <v>209518027.81875</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>14940151970.625</v>
+        <v>219993929.2096876</v>
       </c>
     </row>
     <row r="5">
@@ -1061,19 +1061,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>15378300000</v>
+        <v>161362950</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>16147215000</v>
+        <v>169431097.5</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>16954575750</v>
+        <v>177902652.375</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>17802304537.5</v>
+        <v>186797784.99375</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>18692419764.375</v>
+        <v>196137674.2434376</v>
       </c>
     </row>
     <row r="6">
@@ -1083,19 +1083,19 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-1001699999.999998</v>
+        <v>407214412.5</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>-1051784999.999998</v>
+        <v>427575133.125</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>-1104374249.999998</v>
+        <v>448953889.7812501</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>-1159592962.5</v>
+        <v>471401584.2703126</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-1217572610.625</v>
+        <v>494971663.4838283</v>
       </c>
     </row>
     <row r="9">
@@ -1112,19 +1112,19 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.05010122415000095</v>
+        <v>0.1100281120233391</v>
       </c>
     </row>
     <row r="11">
@@ -1134,19 +1134,19 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>-0.01805006338334623</v>
+        <v>0.08669977141515814</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>-0.01805006338334623</v>
+        <v>0.08669977141515814</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>-0.01805006338334623</v>
+        <v>0.08669977141515814</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>-0.01805006338334626</v>
+        <v>0.08669977141515814</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>-0.01805006338334626</v>
+        <v>0.08669977141515814</v>
       </c>
     </row>
   </sheetData>

</xml_diff>